<commit_message>
chore(sync): update 44 file(s) [.gitignore, CHANGELOG.md, CITATION.cff, data, docs, methodology, outputs, README.md, reviews, scripts, skills]
Automated settle-aware sync of the knowledge base.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/Barotrauma_metrics_reproducibility.xlsx
+++ b/outputs/Barotrauma_metrics_reproducibility.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3250,6 +3250,209 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>1965_Foye</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>1965</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Foye</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Effectsof pressure on survivalofsix species offish</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Live-fish LAB</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>survival vs applied pressure (psi)</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>1988_Davies</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Davies</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>A review of information relating to fish passage through turbines: Implications to tidal power schemes. Journa</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>turbine-passage injury mechanisms (incl. pressure)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>1997_Cada</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Cada</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Shaken, not stirred: the recipe for a fish-friendly turbine</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Review/criteria</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>biological design criteria (pressure)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2001_Perry</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Perry</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Buoyancy compensation of juvenile Chinook salmon implanted with two different size dummy transmitters. Transac</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Lab (buoyancy/physiology)</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>depth/buoyancy compensation</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2023_Koukouvinis</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Koukouvinis</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>State of the Art in Designing Fish-Friendly Turbines - Concepts and Performance Indicators</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>fish-friendly turbine design (pressure)</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3262,7 +3465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S39"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7013,6 +7216,103 @@
       <c r="R39" s="2" t="inlineStr"/>
       <c r="S39" s="2" t="inlineStr"/>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>1965_Foye</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>1965</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Foye</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Effectsof pressure on survivalofsix species offish</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>LAB</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>survival vs applied pressure</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>101–2068 (atm to 300 psi)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>